<commit_message>
test(journey): 第0群を完了し第1群 J10/J11 を実機で消化 (3 → 13 PASS)
第0群 (土台) 12 ステップが全て PASS。第1群も J10-01〜06 / J11-01〜03 を
ブラウザで実操作して消化した。

J10-01 は登録の入力エラー 5 ケース (未入力 / 不正な形式 / 7 文字パスワード /
確認不一致 / 同意なし) を 1 つずつ実行し、20 判定すべて満たすことを確認。
全て日本語で出て英語の既定文は無く、いずれも送信されない。

J10-04 で同意記録の版が現行版 (2026-08-22) と一致することを DB で照会。
ai_training_optin が accepted=false であることも実測した。

J11-02 は「古い更新用トークンも通らない」を検証しようとして、password
サインインが refresh token を発行していないことが分かった。試せないまま
PASS にはできないので、magic-link 経路で本物を 1 本発行して確かめた。
1 回使うと回転し再利用は 401、サインアウト (204) の後も 401。GAP-209 の
失効は実際に効いている。

password サインインに refresh token が無い件は既にバックログにある既知項目
なので、新規に起票せず実測値を追記した。

証拠: .qa/e2e-journey/evidence-20260826/ (J10-03 / J10-06 / J11-01〜03)

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>16%</t>
         </is>
       </c>
     </row>
@@ -2422,11 +2422,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>84%</t>
         </is>
       </c>
     </row>
@@ -7455,14 +7455,19 @@
           <t>手動補正なしでサインインが成立する。seed が必須項目 (パスワード等) を落としていない</t>
         </is>
       </c>
-      <c r="K5" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J00-04_*.png</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>場所=cloud / seed 済み DB では原理的に出ないバグ</t>
+          <t>seed のみの DB (migration 99 + seed 1・users 0) で、DB を手で触らずに登録 → サインアウト → 入り直しが成立。両方とも /projects に着地し JS エラー 0。なお seed にアカウント行は無い (運営固定データのみ) ため、判定は「手動補正なしで入れるか」で行った</t>
         </is>
       </c>
     </row>
@@ -8010,14 +8015,19 @@
           <t>各ケースで日本語のエラーが出て送信されない。英語の既定メッセージが出ない</t>
         </is>
       </c>
-      <c r="K14" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J10-01_*.png</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-210</t>
+          <t>5 ケース (未入力 / 不正な形式のメール / 7 文字パスワード / 確認不一致 / 同意なし) を実操作。20 判定すべて PASS — 全て日本語で出て、英語の既定文は無く、いずれも送信されない</t>
         </is>
       </c>
     </row>
@@ -8070,14 +8080,14 @@
           <t>サーバーが拒否する。画面だけの防御になっていない</t>
         </is>
       </c>
-      <c r="K15" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>画面の検証を回避し fetch で 3 パターン直接投稿 (同意ゼロ / 規約だけ / accepted=false)。すべて 422 で拒否 = 画面だけの防御ではない。この最中に GAP-222 (検証エラーが送信したパスワードを返す) を発見し修正済み</t>
         </is>
       </c>
     </row>
@@ -8132,14 +8142,19 @@
           <t>登録が通り、サインイン画面から抜けて中の画面に着地する</t>
         </is>
       </c>
-      <c r="K16" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K16" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J10-03_after-signup.png</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>正しく入力して登録 → /projects に着地。エラー無し</t>
         </is>
       </c>
     </row>
@@ -8193,14 +8208,14 @@
           <t>記録された版が現行版と一致する。登録日など別の値になっていない</t>
         </is>
       </c>
-      <c r="K17" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-210</t>
+          <t>consents を DB で照会。terms_of_service / privacy_policy とも記録が 2026-08-22 で、legal_documents の現行版と一致。登録日ではない。ai_training_optin は accepted=false (AI 学習デフォルト OFF を実測で確認)</t>
         </is>
       </c>
     </row>
@@ -8253,14 +8268,19 @@
           <t>サイドバー・検索・通知など、押しても何も起きない導線が出ていない</t>
         </is>
       </c>
-      <c r="K18" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K18" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J10-03_after-signup.png</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-207</t>
+          <t>ワークスペース 0 件の状態で、可視の a/button を全走査。href も type=button も無い『押しても何も起きない』要素は 0。サイドバー・検索・通知は그 時点では描画されない (行き止まりの入口を出さない設計)</t>
         </is>
       </c>
     </row>
@@ -8313,14 +8333,19 @@
           <t>再読み込みせずにサイドバーとワークスペース名が出る</t>
         </is>
       </c>
-      <c r="K19" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J10-06_workspace-created.png</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-207</t>
+          <t>名前を入れて作成 → DB に 1 件、画面にワークスペース名とサイドバー (プロジェクト/AI社員/ナレッジ/テンプレート/承認待ち/WS設定) が URL 遷移なしで出る。JS エラー 0</t>
         </is>
       </c>
     </row>
@@ -8374,14 +8399,19 @@
           <t>サインイン画面に着地し、cookie と手元の文脈が消える</t>
         </is>
       </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K20" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J11-01_*.png</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-209</t>
+          <t>アバター → メニューに『プロフィール / サインアウト』。押すと /signin に着地し atelier_access cookie が消える</t>
         </is>
       </c>
     </row>
@@ -8435,14 +8465,19 @@
           <t>サインインへ戻される。古いトークンも通らない</t>
         </is>
       </c>
-      <c r="K21" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J11-02_blocked.png</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-209</t>
+          <t>①中の URL 直接アクセス → /signin?redirect=%2Fprojects に戻される (実機) ②古い更新用トークン: password サインインは refresh token を発行しないため、magic-link 経路で本物を 1 本発行して検証した。(a) 1 回使うと回転し同じトークンの再利用は 401 (b) サインアウト(204)の後は同じトークンが 401。文言も日本語。**password サインインで refresh token が発行されない件は別途 GAP として記録**</t>
         </is>
       </c>
     </row>
@@ -8496,14 +8531,19 @@
           <t>作ったものが残っている</t>
         </is>
       </c>
-      <c r="K22" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J11-03_after-resignin.png</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>同じメール/パスワードで入り直し、作った『通し検証ワークスペース』が画面に残っていることを確認</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): 第1群を完了 (13 → 18 PASS)
J12-01〜03 (再同意の帯) と J13-01/02 (パスワード再設定) を実機で消化した。

J12 は法務文書の現行版を 2026-09-01 に差し替えて帯が出ることを確認し、
本文を読んでから同意すると帯が消え再読み込みでも出ないこと、consents が
1 → 2 に増えて旧版の行が残ることを DB で確かめた。帯を閉じた記録は
localStorage に版つきで保存され、版をさらに上げると再表示される。

J13 は GAP-223 の修正後に実機で最後まで通した。旧パスワード 200 →
再設定 200 → 新パスワード 200 → 旧パスワード 401 → 同じリンクの再利用
401。再設定前の更新用トークンも再設定後は 401。

同意しないまま使い続けられる期間に上限を設けるかは法務判断なので、
判断せずワークブックの注記に残した。

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>22%</t>
         </is>
       </c>
     </row>
@@ -2422,11 +2422,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>78%</t>
         </is>
       </c>
     </row>
@@ -8597,14 +8597,19 @@
           <t>「更新しました。同意をお願いします」の帯が出る</t>
         </is>
       </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J12-01_banner.png</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-206</t>
+          <t>現行版を 2026-09-01 に差し替えてサインイン → 「利用規約を更新しました。内容をご確認のうえ、同意をお願いします。」の帯が実機で出る</t>
         </is>
       </c>
     </row>
@@ -8658,14 +8663,19 @@
           <t>帯が消え、再読み込みしても出ない。旧版の記録は消えず新版が増える</t>
         </is>
       </c>
-      <c r="K24" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J12-02_*.png</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-206</t>
+          <t>「利用規約を読む」で改訂本文 (2026-09-01 の目印入り) を確認 → 戻って「同意する」→ 帯が消え、再読み込みでも出ない。consents は 1 → 2 に増え旧版の行は残る。最新の同意が新版</t>
         </is>
       </c>
     </row>
@@ -8719,14 +8729,19 @@
           <t>同意していない扱いのまま。版が変わればまた出る</t>
         </is>
       </c>
-      <c r="K25" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J12-03_*.png</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>帯を閉じても consents は増えない (2 → 2)。閉じた記録は localStorage に atelier.reconsent.dismissed=terms_of_service:2026-09-02 として版つきで保存され、版を 2026-09-03 に上げると帯が再表示される。**同版のまま再読み込みしても再表示はされない** — 正本の期待は「版が変わればまた出る」なのでこれで満たすが、同意しないまま使い続けられる期間に上限を設けるかは法務判断として残す</t>
         </is>
       </c>
     </row>
@@ -8780,14 +8795,14 @@
           <t>新しいパスワードでサインインでき、古いパスワードでは入れない</t>
         </is>
       </c>
-      <c r="K26" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — 再設定メールが送られず (平文トークンを捨てていた)、利用者は永久に復旧できなかった (GAP-223)。修正後、メールを捕まえて実際に通した: 旧パスワード 200 → 再設定 200 → 新パスワード 200 → 旧パスワード 401 → 同じリンクの再利用 401</t>
         </is>
       </c>
     </row>
@@ -8840,14 +8855,14 @@
           <t>通らない。パスワードを変えたのに古いセッションが生き続けない</t>
         </is>
       </c>
-      <c r="K27" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-209 で見つけた回帰</t>
+          <t>再設定前に発行しておいた更新用トークンで再取得を試み、401 (サインインの有効期限が切れています) を確認。パスワードを変えたのに古いセッションが生き続けることはない</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): 第2群 R-T08 を完了 (21 → 30 PASS)
第2群 (クライアント別 JWT 完全分離) の 9 本を実機で消化。

  J20-01 招待を発行する            (既済)
  J20-02 クライアントが招待リンクで入る  — 別系統の cookie を確認
  J20-03 同意しないと入れない
  J21-01 自分の案件だけ見える        — 社内専用の語が 1 つも出ない
  J22-01 他人の案件へ越境できない     — 参照・投稿・一覧・概要すべて 403/404
  J22-02 クライアント券で社内 API を叩けない — 5 経路すべて 401
  J23-01 クライアントがコメントする
  J23-02 社内側に誰のものか分かる形で届く
  J24-01 期限切れの招待は使えない
  J24-02 失効させると入れない

J22-01 は最初、投稿の payload を誤って 422 (形式検査で弾かれた) になっており、
「拒否された」ように見えていたので作り直した。認可を証明するには、先に
**通る操作があること**を示す必要がある (自分の成果物へのコメント 201)。
全部拒否なら、それは認可ではなく単に壊れている可能性がある。

この通しで見つけた 3 件は別 commit で修正済 (GAP-225 / 226 / 227)。

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>37%</t>
         </is>
       </c>
     </row>
@@ -2391,9 +2391,6 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>0%</t>
@@ -2406,9 +2403,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>0%</t>
@@ -2422,11 +2416,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>63%</t>
         </is>
       </c>
     </row>
@@ -2435,9 +2429,6 @@
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -8916,14 +8907,19 @@
           <t>招待が一覧に出て、リンクが得られる</t>
         </is>
       </c>
-      <c r="K28" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J20-01_*.png</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — RLS の仮の蓋が復活していて発行が 500、一覧もオーナー本人から 0 件だった (GAP-224)。修正後、案件 → 設定 → クライアント招待 の実導線をたどって発行し、DB 1 件・一覧表示・招待リンク表示まで確認</t>
         </is>
       </c>
     </row>
@@ -8980,12 +8976,17 @@
       </c>
       <c r="K29" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J20-02_portal-in.png</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08</t>
+          <t>クライアント招待リンク → 表示名 + 2 種の同意 → ポータルに入室。cookie は atelier_client_access で、社内用 atelier_access とは別名・別系統 (R-T08)</t>
         </is>
       </c>
     </row>
@@ -9040,12 +9041,17 @@
       </c>
       <c r="K30" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J20-03_no-consent.png</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>同意にチェックせず送信 → 拒否。文言は日本語「内容をご確認のうえ、同意にチェックを入れてください。」</t>
         </is>
       </c>
     </row>
@@ -9100,12 +9106,17 @@
       </c>
       <c r="K31" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J21-01_own-project.png</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08</t>
+          <t>自分の案件 (通し案件A) の内容が読める。原価/内部メモ/他案件名/監査ログ/AI社員/タスクボードのいずれも画面に出ない</t>
         </is>
       </c>
     </row>
@@ -9161,12 +9172,17 @@
       </c>
       <c r="K32" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J22-01_cross-project-redo.png</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08 致命級。ここが破れたら公開不可</t>
+          <t>当初は投稿の payload を誤り 422 (= 認可ではなく形式検査で弾かれた) だったため作り直した。**先に「通る操作」を確かめてから拒否を見る**: 自分の成果物へのコメントは 201。その上で他人の案件 (通し案件B) は参照 403 / コメント 403 / 成果物一覧 403 / モック一覧 403 / 概要 403、自分の URL に他人の target を混ぜると 404 (存在ごと秘匿)。画面から直接 /portal?project=&lt;B&gt; を開いても「このプロジェクトを参照する権限がありません。」のみで、応答本文・画面のどちらにも他人の案件名が 1 文字も出ない</t>
         </is>
       </c>
     </row>
@@ -9221,12 +9237,17 @@
       </c>
       <c r="K33" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J22-02_client-token-on-internal.png</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08</t>
+          <t>クライアント券で社内 5 経路 (/me, /workspaces, /projects, /admin/audit-logs, /ai-employees) → すべて 401。当初は本文が英語 (client portal token is not valid here) だったため GAP-225 として起票・修正し、再測定で全 5 本が日本語</t>
         </is>
       </c>
     </row>
@@ -9281,12 +9302,17 @@
       </c>
       <c r="K34" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J23-01_client-comment.png</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>クライアントが成果物にコメント → 201。自分の一覧 (GET /client/projects/{id}/comments) に同じ本文が出る</t>
         </is>
       </c>
     </row>
@@ -9341,12 +9367,17 @@
       </c>
       <c r="K35" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J23-02_internal-and-client-authors.png</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — 社内側の /comments は author_invitation_id (UUID) しか返さず、画面は全員「クライアント（招待）」「メンバー 8f3bbf48」としか出せなかった (= 誰の発言か区別できない)。GAP-226 として起票・修正。再測定: 同じ成果物に 3 件「通しクライアントA（クライアント）: 越境テスト」「通しクライアントA（クライアント）: J23 通しコメント…」「owner-j10: 社内から返信します…」</t>
         </is>
       </c>
     </row>
@@ -9401,12 +9432,17 @@
       </c>
       <c r="K36" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J24-01_expired.png</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期限切れの招待リンク → 入れない (クライアント用 cookie が発行されない)。「招待の有効期限が切れています。再発行を依頼してください。」と日本語。注: expires_at には check 制約 (created_at &lt; expires_at &lt;= created_at+30日) があるため、期限切れを作るには created_at ごと過去へずらす必要がある</t>
         </is>
       </c>
     </row>
@@ -9462,12 +9498,17 @@
       </c>
       <c r="K37" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J24-02_revoked.png</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — 失効させても**配布済みの券が 24h 通り続けた** (失効前 200 → 失効直後も 200)。GAP-227 として起票・修正 (毎リクエストで招待の状態を見る)。再測定: 失効前 200 → 失効直後 401「この招待は取り消されています…」。リンクからの再入場も不可</t>
         </is>
       </c>
     </row>
@@ -9521,14 +9562,19 @@
           <t>一覧に出て、開ける</t>
         </is>
       </c>
-      <c r="K38" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K38" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J30-01_*.png</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>新規プロジェクトから 2 件 (通し案件A / 通し案件B) を作成。DB に各 1 件、一覧にも両方出る</t>
         </is>
       </c>
     </row>
@@ -9581,14 +9627,19 @@
           <t>9 工程が並び、先頭が進行中になっている</t>
         </is>
       </c>
-      <c r="K39" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K39" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J30-02_project-open.png</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>一覧のカード (button) を押して /projects/dashboard?project=... に遷移。phases テーブルに 9 工程。タブは ダッシュボード/工程/タスク/進行/議事録/スケジュール/営業ドラフト/モック/取り込み/シークレット/設定</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): 第3群前半 J30〜J32 を消化 (30 → 37 PASS)
  J30-03 工程を進める — 承認 → 次工程開始の 2 ボタンを実クリック、DB 突合
  J30-04 確定した工程が凍結される — 凍結前は変えられることを先に確認し、
         確認なし確定 403 / confirm 確定 200 / 凍結後の変更・削除 409
  J31-01 メンバーを招待する (GAP-229 修正後に PASS)
  J31-02 メンバーが入って作業できる
  J31-03 メンバーは権限外の操作をできない — owner 専用 3 操作すべて 403。
         認可を突くには登録済みメールを使う (未登録だと 422 が先に出る)
  J32-01 承認待ちを承認する (GAP-230 修正後に PASS)
  J32-02 承認待ちを却下する — rejected/blocked として承認と区別できる

この区間で見つけた 3 件は別 commit で修正済 (GAP-228 / 229 / 230)。

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>45%</t>
         </is>
       </c>
     </row>
@@ -2416,11 +2416,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>63%</t>
+          <t>55%</t>
         </is>
       </c>
     </row>
@@ -9694,12 +9694,17 @@
       </c>
       <c r="K40" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J30-03_next-started.png</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>S-F01 で「この工程を完了として承認」→「次工程（要件定義）を開始」を実クリック。DB: ヒアリング=completed / 要件定義=in_progress。承認と開始が別ボタンなのは二重進行防止の設計 (GAP-031②)</t>
         </is>
       </c>
     </row>
@@ -9754,12 +9759,17 @@
       </c>
       <c r="K41" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J30-04_frozen-final.png</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>凍結前に meta_tags を変えられることを先に確認 (200・DB 反映) → 確認なし確定 403 (明示の操作が要る) → confirm つき確定 200 (DB=frozen・次フェーズが active に) → 凍結後の変更 409・削除 409、DB は 1 文字も変わらず。準備中に GAP-228 (同名モック作成が 500) を発見・修正</t>
         </is>
       </c>
     </row>
@@ -9814,12 +9824,17 @@
       </c>
       <c r="K42" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J31-01_invited.png</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 500「サーバーでエラーが発生しました」— RLS ポリシーの自己参照再帰で**メンバー招待が全滅**していた。GAP-229 として起票・修正 (t-d-14 の owner 判定を SECURITY DEFINER 関数へ / 再適用パスによる「復活」も根治)。再測定: member-j31 を実登録 → S-A03 メンバータブから招待 → 一覧に 2 人目が出て DB に membership (role=member)</t>
         </is>
       </c>
     </row>
@@ -9875,12 +9890,17 @@
       </c>
       <c r="K43" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J31-02_member-projects.png</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>member-j31 でサインイン → 参加した WS のプロジェクト一覧に通し案件A/B が見える。API も 200</t>
         </is>
       </c>
     </row>
@@ -9935,12 +9955,17 @@
       </c>
       <c r="K44" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J31-03_member-settings.png</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>member で owner 専用 3 操作 (メンバー招待/WS 名変更/WS 削除) → すべて 403 + 日本語。DB 無変化。設定画面は白画面にならない。注: 招待の認可を突くには**登録済みメール**を使う (未登録だと 422 が先に出る)</t>
         </is>
       </c>
     </row>
@@ -9996,12 +10021,17 @@
       </c>
       <c r="K45" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J32-01_approved.png</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — インボックスで承認しても inbox の行だけ approved で**タスクは awaiting のまま** (幽霊承認)。GAP-230 として起票・修正 (decide がタスク本体へ伝播)。再測定: 承認 → 一覧から消え、inbox=approved / task=done。注: 承認待ちの生産側 (AI 実行完了 → awaiting) は Bridge = Mac 側なので、ここでは awaiting 状態を seed して消費側を通した</t>
         </is>
       </c>
     </row>
@@ -10056,12 +10086,17 @@
       </c>
       <c r="K46" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J32-02_rejected.png</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>却下 → inbox=rejected / task=blocked + 理由。承認済み (approved/done) と明確に区別できる</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): J34 議事録 / J35 ナレッジを消化 (37 → 43 PASS + 1 BLOCKED)
  J34-01 音声アップロード — 実 WAV (espeak-ng 合成) を署名付き URL に PUT。
         storage は Supabase Storage 互換のローカル・ハーネス (製品コード無改変)。
         発見: ATELIER_SUPABASE_ADMIN_API_URL は storage と auth の両方を
         切り替える 1 つの env (本番は同一ホストなので設計どおり)
  J34-02 文字起こし — worker 1 巡で実 faster-whisper (small) が処理。
         喋った内容が画面に一字一句出た。日本語 TTS は音声品質が低く
         whisper が拾えないため検証は英語音声 (製品は言語自動判定で同経路)
  J34-03 採用 — 構造化解析は本人サブスク (Bridge) = Mac 側のため BLOCKED。
         解析前の正直な断り (409・日本語) は確認済み
  J35-01 ナレッジ 作成→編集→削除 (論理削除・復活しない)
  J35-02 検索 (GAP-231 修正後に PASS)
  J35-03 別アカウントのナレッジは検索に出ない
  J35-04 候補の採用/却下 — 採用だけが正式ナレッジになる

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>52%</t>
         </is>
       </c>
     </row>
@@ -2403,9 +2403,12 @@
           <t>BLOCKED</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1%</t>
         </is>
       </c>
     </row>
@@ -2416,11 +2419,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>46%</t>
         </is>
       </c>
     </row>
@@ -10334,12 +10337,17 @@
       </c>
       <c r="K50" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J34-01_uploaded.png</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>実 WAV (espeak-ng で合成した会議音声・約 20 秒) を S-M01 で選択 → 署名付き URL に PUT。external_uploads に行、storage に実体。storage は Supabase Storage 互換のローカル・ハーネス (製品コードは無改変・実契約どおりの口)。準備中の発見: ATELIER_SUPABASE_ADMIN_API_URL は storage と auth の両方を切り替える 1 つの env (本番は同一ホストなので設計どおり) — ハーネスにも GoTrue 互換の口が要る</t>
         </is>
       </c>
     </row>
@@ -10394,12 +10402,17 @@
       </c>
       <c r="K51" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J34-02_transcript.png</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>worker を 1 巡実行 → **実 faster-whisper (small)** が文字起こし。DB: parsed_at 打刻・parse_error なし。画面で本文が読める — 実際に喋った「delivery date will be the 15th of next month / Friday at 3 PM」が一字一句出た。注: 日本語 TTS (espeak-ng + mbrola-jp1) は音声品質が低く whisper が拾えないため検証は英語音声。製品は言語自動判定で日本語も同経路</t>
         </is>
       </c>
     </row>
@@ -10454,12 +10467,17 @@
       </c>
       <c r="K52" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J34-02_transcript.png</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>採用候補は**構造化解析 (9 セクション) の結果**から出る。解析は本人サブスク (Bridge) 経路の LLM 実行 = Mac 側。この環境では解析前の正直な断りを確認済み — GET adoptable が 409「いまは採用できません。解析を実行してからお試しください。」(日本語・嘘の成功を出さない)。解除条件: Mac で Bridge を接続し「解析を再開」→ 採用まで一周</t>
         </is>
       </c>
     </row>
@@ -10514,12 +10532,17 @@
       </c>
       <c r="K53" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J35-04_candidates.png</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>作成 201 → 編集反映 (一覧にも) → 削除 204 → 一覧から消え、DB は論理削除。復活しない</t>
         </is>
       </c>
     </row>
@@ -10574,12 +10597,17 @@
       </c>
       <c r="K54" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J35-04_candidates.png</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>当初 FAIL — 意味検索に足切りが無く、デタラメな語でも最近傍 3 件が返った (類似 0.74〜0.80)。GAP-231 として起票・修正 (足切り 0.83)。再測定: 該当語 0.951/0.897 でヒット、デタラメ語 2 種 → 0 件</t>
         </is>
       </c>
     </row>
@@ -10635,12 +10663,17 @@
       </c>
       <c r="K55" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J35-04_candidates.png</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08</t>
+          <t>別アカウント (member-j31 の user スコープ) に同じ固有語を含むナレッジを作成 → owner の検索に 1 件も出ない</t>
         </is>
       </c>
     </row>
@@ -10695,12 +10728,17 @@
       </c>
       <c r="K56" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>.qa/e2e-journey/evidence-20260826/J35-04_after.png</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>候補 2 件 (生産側は AI 会話 = Bridge なので seed) → 採用は approved + 正式ナレッジ 1 件、却下は rejected でナレッジにならない。画面 S-K01 に採用/却下ボタンが候補ごとに出ている</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): J02 運営テンプレ/スキル・J03 法務改訂・J40 Bridge 未接続を消化 (43 → 50 PASS + 2 BLOCKED)
- J02-01/02/03: テンプレ編集が DB 反映 (version 1→2)・スキル装着・
  スキル本文の秘匿 (先に admin で読めることを示してから一般 403 +
  DB 直読 permission denied) を実測。追加/削除の口は仕様として無く
  7 人の既定テンプレを編集するモデル (GAP-031⑤/T-A-42)
- J03-01: 版付き SQL の正規手順で規約を改訂 → 現行 1 件は部分一意
  index が強制 (二重 current は拒否を実測)、旧版残存。QA 版は復元済
- J03-02: ゲストで改訂版が公開ページに即時反映されることを確認。
  特商法の（担当者名）のみ経営者の実名待ち (既知・go-no-go 条件)。
  改訂で再同意バナーが出る連鎖も確認
- J40-01: 実送信で「ローカル実行 (Bridge) がオフライン…」の正直な
  案内 + 常時チップ + 接続フロー。未設定と混同しない
- J40-03: 実行前に「自分の Claude プランで実行・追加の従量課金は
  発生しません」を確認できる
- J40-02 は BLOCKED (Bridge + 本人サブスクが要る / Mac で実施)

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2340,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>61%</t>
         </is>
       </c>
     </row>
@@ -2404,11 +2404,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>2%</t>
         </is>
       </c>
     </row>
@@ -2419,11 +2419,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>37%</t>
         </is>
       </c>
     </row>
@@ -2451,6 +2451,8 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7702,12 +7704,17 @@
       </c>
       <c r="K9" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>J02_admin-home.png ほか / DB: jarvis specialty更新 version1→2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>場所=cloud / 「整備済みを確認」で済ませず実際に 1 件回す</t>
+          <t>編集は API PATCH → 一覧・DB 反映を実測 (version 自動increment)。追加/削除の口は仕様として存在しない — 7 人の既定テンプレを編集するモデル (GAP-031⑤/T-A-42、PATCH 可能項目にも is_active 無し)。期待結果は製品設計に照らして判定</t>
         </is>
       </c>
     </row>
@@ -7764,12 +7771,17 @@
       </c>
       <c r="K10" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>API: skill create 201 (version必須) → attach 200 → list に装着反映</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>スキル追加→ジャービスに装着→一覧で装着状態を確認 (実測)</t>
         </is>
       </c>
     </row>
@@ -7825,12 +7837,17 @@
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>API 403「この操作は運営のみが行えます。」/ DB: permission denied for table skills</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T06</t>
+          <t>先に admin で読めることを確認してから一般利用者で拒否を実測 (GAP-144 列 revoke)。合言葉「ゴールデンレトリバー割引」は画面/配布 JS/一般 API のどこにも出ない</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7904,17 @@
       </c>
       <c r="K12" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>psql: 改訂後 current=1/7 版・旧版残存・二重 current は legal_documents_current_uidx が拒否 (実測 ERROR)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>場所=cloud / 順序を誤ると一意制約で失敗する</t>
+          <t>改訂は版付き SQL が正規の運用経路 (管理 UI は仕様として無い / gap-208 等の migration がその実例)。手順=先に current を降ろす→新版 insert。検証後に QA 版 (2026-09-04) を削除し 2026-09-03 現行へ復元 (G-10 副作用復帰)</t>
         </is>
       </c>
     </row>
@@ -7947,12 +7969,17 @@
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>J03_terms-new-version.png / J03_tokushoho.png — ゲストで改訂版 (第16条/2026-09-04) を確認</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>公開ページは正本 API を都度取得 (キャッシュ滞留なし)。実額 5,000 円の記載あり。特商法の運営統括責任者（担当者名）のみ経営者の実名待ち (既知・go-no-go 条件、AI が勝手に埋めない方針)。改訂により利用者側へ再同意バナーが出ることも確認 (GAP-206 連鎖)</t>
         </is>
       </c>
     </row>
@@ -10793,12 +10820,17 @@
       </c>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>J40_chat-send-offline.png — 実送信で「ローカル実行 (Bridge) がオフラインのため応答できません。お使いの PC で Bridge を起動してから再送してください。」</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-168/206</t>
+          <t>ヘッダーに常時「プラン未接続 — ここから接続」チップ + クリックで接続フロー。未設定との混同なし (X-Atelier-Reason=bridge_offline のときだけ未接続と案内 / GAP-206 是正)。「時間をおいて」も出ない</t>
         </is>
       </c>
     </row>
@@ -10853,12 +10885,17 @@
       </c>
       <c r="K58" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: Bridge (Electron) と本人の Claude サブスクが要る。解除条件: Mac で Bridge を起動→チャットの「ここから接続」→接続トークン発行→アプリで接続→表示が「接続中」になること</t>
         </is>
       </c>
     </row>
@@ -10913,12 +10950,17 @@
       </c>
       <c r="K59" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>J40_connect-flow.png — 「自分の Claude プランで実行 / あなたのパソコンを経由して、あなたの Claude 月額プランの範囲内で実行されます。追加の従量課金は発生しません。」</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-178</t>
+          <t>実行前に常時チップ (接続状態) + 1 クリックで経路と費用の帰属を確認できる。コンポーザにも「PC 操作: なし」と「外部の学習には使いません」を常時表示</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(journey): 第4群後半〜最終群を消化 — 通し 82 本の判定が全て確定 (61 PASS / 21 BLOCKED / 0 TODO)
- J43-03: 実行が失敗しても打った文章は消えない (先に永続化・失敗理由も
  スレッドに残る。DB 突合 + ブラウザ開き直しで実測)
- J33-02: 壊れた/非対応ファイルは黙って捨てられない (成功 2/失敗 1 を
  明示、per-file の理由「対応していない形式です」)
- J50-01/02・J51-02: BLOCKED — Stripe テストモード実鍵が要る (G3:
  決済の実副作用はモックで PASS にしない)。誠実 degrade
  「決済連携が未設定です」と表示層 (pro 状態の請求期間表示) は実測済
- J51-01: 解約条件 (期間末まで利用可・日割り返金なし) が押す前に読める
- J51-03: free に解約の死にボタンなし
- J60-01/02: 混雑実績 (machine 横断・90 日) と「あと何台増やせるか」が
  運営画面で読める (実データ)
- J61-01/02: 監査ログで誰が何をしたか追える / R-T08 越境試験 —
  先に通る側 (自 WS 4 行・自分の行 13 行) を示してから、他テナント 0 行・
  非 admin 403 を実測。update/delete は全面禁止
- 残る 16 本 (J01/J33-01,03/J41/J42/J43-01,02) は BLOCKED —
  Bridge + 本人の Claude サブスク (Mac) が要る。理由と解除条件を各行に記録

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/.qa/e2e-journey/journey-20260825.xlsx
+++ b/.qa/e2e-journey/journey-20260825.xlsx
@@ -2377,11 +2377,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>74%</t>
         </is>
       </c>
     </row>
@@ -2404,11 +2404,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>26%</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2418,9 @@
           <t>TODO</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>30</v>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2444,7 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>NO (BLOCKED 残)</t>
         </is>
       </c>
     </row>
@@ -7520,12 +7517,17 @@
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: Bridge + 本人 Claude サブスクでの既定デザインテンプレ生成が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -7581,12 +7583,17 @@
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: J01-01 の成果 (既定テンプレ) が前提。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -7643,12 +7650,17 @@
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: J01-01/02 の成果が前提。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -10182,12 +10194,17 @@
       </c>
       <c r="K47" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: 取り込み後の工程提案は AI 解析 (本人サブスク経路) を含む。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -10242,12 +10259,17 @@
       </c>
       <c r="K48" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>J33_import-results.png — 成功 2 / 失敗 1、j33-data.xyz「対応していない形式です」を個別表示</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>1 ファイルの失敗で全体を落とさず per-file の理由が出る。中身が壊れた .xlsx はファイル成果物として保存される (取り込み時は形式検証せず、開く時に誠実エラー — GAP-176 系)。黙って捨てられるファイルは無い</t>
         </is>
       </c>
     </row>
@@ -10303,12 +10325,17 @@
       </c>
       <c r="K49" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: J33-01 の提案結果が前提。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11016,12 +11043,17 @@
       </c>
       <c r="K60" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: チャット応答 = 本人の PC の Bridge + 本人サブスクで実行。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11077,12 +11109,17 @@
       </c>
       <c r="K61" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: 同上 (応答内容の検証)。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11138,12 +11175,17 @@
       </c>
       <c r="K62" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: 同上 (3 ターン以上の会話)。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11199,12 +11241,17 @@
       </c>
       <c r="K63" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-139</t>
+          <t>この環境では実施不可: 同上 + GAP-139 成果物自動仕分けは実応答が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11259,12 +11306,17 @@
       </c>
       <c r="K64" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-147 回帰</t>
+          <t>この環境では実施不可: 同上 + GAP-147 部分改訂は実 LLM 応答が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11320,12 +11372,17 @@
       </c>
       <c r="K65" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-161</t>
+          <t>この環境では実施不可: 同上 + GAP-161 添付参照は実 LLM 応答が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11381,12 +11438,17 @@
       </c>
       <c r="K66" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-130</t>
+          <t>この環境では実施不可: PC 操作の承認モード (GAP-130) は Bridge 実機が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11442,12 +11504,17 @@
       </c>
       <c r="K67" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: 同上。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11503,12 +11570,17 @@
       </c>
       <c r="K68" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>この環境では実施不可: 同上。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11564,12 +11636,17 @@
       </c>
       <c r="K69" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-203</t>
+          <t>この環境では実施不可: 混雑の実測は複数実行 (Bridge 実機) が要る。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11625,12 +11702,17 @@
       </c>
       <c r="K70" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>場所=mac / GAP-203 回帰</t>
+          <t>この環境では実施不可: 同上 (順番待ち中の切断)。解除条件: Mac で Bridge を起動し本人の Claude サブスクで実行 (反映手順は Mac 反映コマンドで main へ)</t>
         </is>
       </c>
     </row>
@@ -11685,12 +11767,17 @@
       </c>
       <c r="K71" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>J43_after-failure.png / J43_reopen-thread.png — 失敗直後も文章が残り、ブラウザを閉じて開き直しても残る (DB chat_messages に実在)</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>送信は先に永続化され、実行失敗 (Bridge オフライン) の理由もスレッドに残る</t>
         </is>
       </c>
     </row>
@@ -11746,12 +11833,17 @@
       </c>
       <c r="K72" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>J50_plan-free-unconfigured.png — 鍵なし環境では「決済連携が未設定です」を明示し偽の申込導線を出さない (誠実 degrade は実測 PASS)</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>実施不可: Stripe テストモードの実鍵 (sk_test) が要る (G3: 決済の実副作用はモックで PASS にしない)。解除条件: STRIPE_SECRET_KEY/STRIPE_WEBHOOK_SECRET (テストモード) を設定した環境で checkout 実走 → Stripe 側の subscription 状態を実 API で照会</t>
         </is>
       </c>
     </row>
@@ -11806,12 +11898,17 @@
       </c>
       <c r="K73" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>J51_plan-pro-cancel-terms.png — 表示層は検証済 (billing 行が pro なら請求期間・プラン章票が出る)</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>実施不可: 「申込 → 反映」の本体は Stripe checkout/webhook 経由の workspace_billing 更新で、実鍵が要る。表示層のみ内部状態を模して検証済。解除条件は J50-01 と同じ</t>
         </is>
       </c>
     </row>
@@ -11866,12 +11963,17 @@
       </c>
       <c r="K74" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>J51_plan-pro-cancel-terms.png — 「解約後も、いまの請求期間の終わりまではご利用いただけます。日割りでの返金はありません。」がボタンを押す前に読める + 「現在の請求期間: …まで」表示</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-208</t>
+          <t>GAP-208 の解約導線。契約者 (pro) には「プランの管理・解約」の口が必ず出る (申し込めるのに解約できない状態を作らない)</t>
         </is>
       </c>
     </row>
@@ -11926,12 +12028,17 @@
       </c>
       <c r="K75" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-208</t>
+          <t>実施不可: 解約の実行は Stripe カスタマーポータルで行われ、実鍵と Stripe 側状態の照会が要る (G3)。解除条件: sk_test 環境でポータル遷移 → 解約 → subscription.status=canceled を実 API で確認 → 画面が free に戻ること</t>
         </is>
       </c>
     </row>
@@ -11986,12 +12093,17 @@
       </c>
       <c r="K76" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>J50_plan-free-unconfigured.png — free 状態に解約ボタンは存在しない (0 個)。未設定環境では「決済連携が未設定です」を明示</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>死にボタンなし。存在しない契約に対する解約 UI を出さない</t>
         </is>
       </c>
     </row>
@@ -12046,12 +12158,17 @@
       </c>
       <c r="K77" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>J52_deletion-receipt-real.png — 誤 pw 401「パスワードが正しくありません。」→ 正 pw で受付 + DB: deleted_at 立つ (purge 対象化)。受付に実際の削除予定日時</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>GAP-233 を発見・修正して PASS。従来は監査記録のみkeyで deleted_at が立たず「30 日後に削除」が嘘だった</t>
         </is>
       </c>
     </row>
@@ -12106,12 +12223,17 @@
       </c>
       <c r="K78" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>J52_restored.png — サインイン画面の「退会済みアカウントの復元」で email+pw → 復元成功 → DB: deleted_at 解除 → サインイン成功</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>GAP-233 で復元導線を新設して PASS (API はあったが UI から実行不能だった)</t>
         </is>
       </c>
     </row>
@@ -12166,12 +12288,17 @@
       </c>
       <c r="K79" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>J52_signin-blocked.png — 退会直後のサインインは「メールアドレスまたはパスワードが違います。」で拒否</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>文言は存在秘匿設計 (退会済みであることを未認証の第三者に漏らさない)。復元は専用導線から</t>
         </is>
       </c>
     </row>
@@ -12226,12 +12353,17 @@
       </c>
       <c r="K80" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>J60_admin-health.png — 「混雑の実績 (machine 横断)」直近 7 日: 混雑なし (全 machine)・延べ待たせた人数・お断り回数</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-208</t>
+          <t>GAP-208。通知は入れない経営者判断のため画面が唯一の観測点。machine 横断の capacity_events 集計 (90 日保持)</t>
         </is>
       </c>
     </row>
@@ -12286,12 +12418,17 @@
       </c>
       <c r="K81" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>J60_admin-health.png — 「増やせる余地 (machine 数)」DB 直結 30×2=60/予算 60 — この予算で 2 台まで。以降は Supavisor 切替 (runbook 参照) と明記</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-205</t>
+          <t>GAP-205。増やそうとした瞬間に壁を知る、を無くす表示</t>
         </is>
       </c>
     </row>
@@ -12347,12 +12484,17 @@
       </c>
       <c r="K82" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>J61_audit-logs.png — 監査ログ画面 (1 年保持・CSV エクスポート・actor 検索)。今日の通しの実操作が actor 付きで並ぶ</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>運営 admin 専用 (非 admin は 403「この操作は運営のみが行えます。」実測)</t>
         </is>
       </c>
     </row>
@@ -12407,12 +12549,17 @@
       </c>
       <c r="K83" s="16" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>SQL: j10 は自 WS の行 4 件が見える (先に通る側) → 別テナント j52 は自分の行 13 件のみ・他 WS の行 0 件・全可視 13 件 / 非 admin の /admin/audit-logs は 403</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>場所=cloud / R-T08</t>
+          <t>R-T08。audit_logs_select = 本人 or 所属 WS のみ。update/delete は全面禁止 (改ざん不可)</t>
         </is>
       </c>
     </row>

</xml_diff>